<commit_message>
Fix Excel example binary
</commit_message>
<xml_diff>
--- a/projects/01-document-automation-toolkit/examples/records.xlsx
+++ b/projects/01-document-automation-toolkit/examples/records.xlsx
@@ -429,4 +429,198 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="50" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="40" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="44" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="26" customHeight="1">
+      <x:c r="A1" s="23" t="str">
+        <x:v>record_id</x:v>
+      </x:c>
+      <x:c r="B1" s="23" t="str">
+        <x:v>document_title</x:v>
+      </x:c>
+      <x:c r="C1" s="23" t="str">
+        <x:v>recipient</x:v>
+      </x:c>
+      <x:c r="D1" s="23" t="str">
+        <x:v>owner</x:v>
+      </x:c>
+      <x:c r="E1" s="23" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="F1" s="23" t="str">
+        <x:v>created_on</x:v>
+      </x:c>
+      <x:c r="G1" s="23" t="str">
+        <x:v>due_on</x:v>
+      </x:c>
+      <x:c r="H1" s="23" t="str">
+        <x:v>summary</x:v>
+      </x:c>
+      <x:c r="I1" s="23" t="str">
+        <x:v>metrics</x:v>
+      </x:c>
+      <x:c r="J1" s="23" t="str">
+        <x:v>risks</x:v>
+      </x:c>
+      <x:c r="K1" s="23" t="str">
+        <x:v>next_steps</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="44" customHeight="1">
+      <x:c r="A2" s="17" t="str">
+        <x:v>PRJ-001</x:v>
+      </x:c>
+      <x:c r="B2" s="17" t="str">
+        <x:v>Quarterly Operations Summary</x:v>
+      </x:c>
+      <x:c r="C2" s="17" t="str">
+        <x:v>Operations Team</x:v>
+      </x:c>
+      <x:c r="D2" s="17" t="str">
+        <x:v>Alex Morgan</x:v>
+      </x:c>
+      <x:c r="E2" s="17" t="str">
+        <x:v>On track</x:v>
+      </x:c>
+      <x:c r="F2" s="28" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="G2" s="28" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+      <x:c r="H2" s="17" t="str">
+        <x:v>A concise summary of operational progress, open decisions and measurable outcomes for the current quarter.</x:v>
+      </x:c>
+      <x:c r="I2" s="17" t="str">
+        <x:v>Items processed=1240;Exceptions reviewed=38;Completion rate=96%</x:v>
+      </x:c>
+      <x:c r="J2" s="17" t="str">
+        <x:v>Supplier response time remains variable;One source file still arrives manually</x:v>
+      </x:c>
+      <x:c r="K2" s="17" t="str">
+        <x:v>Confirm October priorities|Automate the remaining source import|Close the exception backlog</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="44" customHeight="1">
+      <x:c r="A3" s="17" t="str">
+        <x:v>PRJ-002</x:v>
+      </x:c>
+      <x:c r="B3" s="17" t="str">
+        <x:v>Client Data Migration Brief</x:v>
+      </x:c>
+      <x:c r="C3" s="17" t="str">
+        <x:v>Client Success</x:v>
+      </x:c>
+      <x:c r="D3" s="17" t="str">
+        <x:v>Jordan Lee</x:v>
+      </x:c>
+      <x:c r="E3" s="17" t="str">
+        <x:v>Attention required</x:v>
+      </x:c>
+      <x:c r="F3" s="28" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="G3" s="28" t="n">
+        <x:v>46283</x:v>
+      </x:c>
+      <x:c r="H3" s="17" t="str">
+        <x:v>Migration preparation for a synthetic customer dataset. The document records scope, validation points and the next actions without exposing any real client data.</x:v>
+      </x:c>
+      <x:c r="I3" s="17" t="str">
+        <x:v>Rows received=18500;Duplicates flagged=312;Invalid emails=47</x:v>
+      </x:c>
+      <x:c r="J3" s="17" t="str">
+        <x:v>Source B contains inconsistent date formats</x:v>
+      </x:c>
+      <x:c r="K3" s="17" t="str">
+        <x:v>Approve mapping rules|Resolve date ambiguity|Run final import rehearsal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="44" customHeight="1">
+      <x:c r="A4" s="17" t="str">
+        <x:v>PRJ-003</x:v>
+      </x:c>
+      <x:c r="B4" s="17" t="str">
+        <x:v>Automation Delivery Note</x:v>
+      </x:c>
+      <x:c r="C4" s="17" t="str">
+        <x:v>Internal Review</x:v>
+      </x:c>
+      <x:c r="D4" s="17" t="str">
+        <x:v>Sam Patel</x:v>
+      </x:c>
+      <x:c r="E4" s="17" t="str">
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="F4" s="28" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="G4" s="28" t="n">
+        <x:v>46277</x:v>
+      </x:c>
+      <x:c r="H4" s="17" t="str">
+        <x:v>Delivery summary for a small automation that converts structured input into repeatable business documents and records validation failures separately.</x:v>
+      </x:c>
+      <x:c r="I4" s="17" t="str">
+        <x:v>Documents generated=24;Rejected records=2;Automated checks=8</x:v>
+      </x:c>
+      <x:c r="J4" s="17" t="str"/>
+      <x:c r="K4" s="17" t="str">
+        <x:v>Archive the delivery package|Document maintenance steps</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="44" customHeight="1">
+      <x:c r="A5" s="30" t="str">
+        <x:v>INVALID-01</x:v>
+      </x:c>
+      <x:c r="B5" s="30" t="str"/>
+      <x:c r="C5" s="30" t="str">
+        <x:v>Internal Review</x:v>
+      </x:c>
+      <x:c r="D5" s="30" t="str">
+        <x:v>Casey Smith</x:v>
+      </x:c>
+      <x:c r="E5" s="30" t="str">
+        <x:v>Draft</x:v>
+      </x:c>
+      <x:c r="F5" s="31" t="n">
+        <x:v>46271</x:v>
+      </x:c>
+      <x:c r="G5" s="31" t="n">
+        <x:v>46285</x:v>
+      </x:c>
+      <x:c r="H5" s="30" t="str">
+        <x:v>This row intentionally misses a required document title so validation can be demonstrated.</x:v>
+      </x:c>
+      <x:c r="I5" s="30" t="str">
+        <x:v>Rows=1</x:v>
+      </x:c>
+      <x:c r="J5" s="30" t="str"/>
+      <x:c r="K5" s="30" t="str">
+        <x:v>Review input</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cddb29754e34f0b"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
</xml_diff>